<commit_message>
feat: generated 'Contains Duplicate' via AI + removed from sheet (90 remaining)
</commit_message>
<xml_diff>
--- a/Sheets/Deloitte_100_Coding_Questions.xlsx
+++ b/Sheets/Deloitte_100_Coding_Questions.xlsx
@@ -129,39 +129,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -481,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K92"/>
+  <dimension ref="A1:K91"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.421875" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="6.00390625" customWidth="1" min="1" max="1"/>
@@ -565,17 +544,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Kadane's Algorithm</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Contains Duplicate</t>
+          <t>Maximum Subarray</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Easy-Medium</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -585,7 +564,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/contains-duplicate/</t>
+          <t>https://leetcode.com/problems/maximum-subarray/</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -615,17 +594,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Kadane's Algorithm</t>
+          <t>Prefix Product</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Maximum Subarray</t>
+          <t>Product of Array Except Self</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Easy-Medium</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -635,12 +614,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/maximum-subarray/</t>
+          <t>https://leetcode.com/problems/product-of-array-except-self/</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -650,7 +629,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -665,17 +644,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Prefix Product</t>
+          <t>Merging</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Product of Array Except Self</t>
+          <t>Merge Sorted Array</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -685,7 +664,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/product-of-array-except-self/</t>
+          <t>https://leetcode.com/problems/merge-sorted-array/</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -715,12 +694,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Merging</t>
+          <t>Missing Element</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Merge Sorted Array</t>
+          <t>Missing Number</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -735,12 +714,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/merge-sorted-array/</t>
+          <t>https://leetcode.com/problems/missing-number/</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -750,7 +729,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -760,17 +739,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Arrays</t>
+          <t>Mathematics</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Missing Element</t>
+          <t>Digit Manipulation</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Missing Number</t>
+          <t>Armstrong Number</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -780,12 +759,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/missing-number/</t>
+          <t>https://www.geeksforgeeks.org/c-program-to-check-armstrong-number/</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -810,17 +789,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Mathematics</t>
+          <t>Strings</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Digit Manipulation</t>
+          <t>Anagram</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Armstrong Number</t>
+          <t>Valid Anagram</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -830,12 +809,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/c-program-to-check-armstrong-number/</t>
+          <t>https://leetcode.com/problems/valid-anagram/</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -865,12 +844,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Anagram</t>
+          <t>Palindrome</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Valid Anagram</t>
+          <t>Valid Palindrome</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -885,7 +864,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/valid-anagram/</t>
+          <t>https://leetcode.com/problems/valid-palindrome/</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -915,17 +894,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Palindrome</t>
+          <t>Reversal</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Valid Palindrome</t>
+          <t>Reverse Words in a String</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -935,12 +914,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/valid-palindrome/</t>
+          <t>https://leetcode.com/problems/reverse-words-in-a-string/</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -950,7 +929,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -965,12 +944,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Reversal</t>
+          <t>Sliding Window</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Reverse Words in a String</t>
+          <t>Longest Substring Without Repeating Characters</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -985,12 +964,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/reverse-words-in-a-string/</t>
+          <t>https://leetcode.com/problems/longest-substring-without-repeating-characters/</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1000,7 +979,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1015,12 +994,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Sliding Window</t>
+          <t>Compression</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Longest Substring Without Repeating Characters</t>
+          <t>String Compression</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1035,12 +1014,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/longest-substring-without-repeating-characters/</t>
+          <t>https://leetcode.com/problems/string-compression/</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1050,7 +1029,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1065,17 +1044,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Compression</t>
+          <t>Parsing</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>String Compression</t>
+          <t>Roman to Integer</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1085,7 +1064,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/string-compression/</t>
+          <t>https://leetcode.com/problems/roman-to-integer/</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1110,17 +1089,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Strings</t>
+          <t>Number Theory</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Parsing</t>
+          <t>GCD</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Roman to Integer</t>
+          <t>GCD of Two Numbers (Euclidean Algorithm)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1130,17 +1109,17 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/roman-to-integer/</t>
+          <t>https://www.geeksforgeeks.org/c-program-for-basic-euclidean-algorithms/</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1150,7 +1129,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1160,37 +1139,37 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Number Theory</t>
+          <t>Strings</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>GCD</t>
+          <t>Grouping</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>GCD of Two Numbers (Euclidean Algorithm)</t>
+          <t>Group Anagrams</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/c-program-for-basic-euclidean-algorithms/</t>
+          <t>https://leetcode.com/problems/group-anagrams/</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1200,7 +1179,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1215,17 +1194,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Grouping</t>
+          <t>Counting</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Group Anagrams</t>
+          <t>First Unique Character in a String</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1235,7 +1214,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/group-anagrams/</t>
+          <t>https://leetcode.com/problems/first-unique-character-in-a-string/</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1265,12 +1244,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Counting</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>First Unique Character in a String</t>
+          <t>Longest Common Prefix</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1285,7 +1264,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/first-unique-character-in-a-string/</t>
+          <t>https://leetcode.com/problems/longest-common-prefix/</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1310,22 +1289,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Strings</t>
+          <t>HashMap / HashSet</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Frequency</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Longest Common Prefix</t>
+          <t>Top K Frequent Elements</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1335,7 +1314,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/longest-common-prefix/</t>
+          <t>https://leetcode.com/problems/top-k-frequent-elements/</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1365,17 +1344,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Frequency</t>
+          <t>Set Operations</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Top K Frequent Elements</t>
+          <t>Intersection of Two Arrays</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1385,7 +1364,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/top-k-frequent-elements/</t>
+          <t>https://leetcode.com/problems/intersection-of-two-arrays/</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1415,17 +1394,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Set Operations</t>
+          <t>Subarray</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Intersection of Two Arrays</t>
+          <t>Subarray Sum Equals K</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1435,12 +1414,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/intersection-of-two-arrays/</t>
+          <t>https://leetcode.com/problems/subarray-sum-equals-k/</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1450,7 +1429,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1465,12 +1444,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Subarray</t>
+          <t>Sequence</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Subarray Sum Equals K</t>
+          <t>Longest Consecutive Sequence</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1485,12 +1464,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/subarray-sum-equals-k/</t>
+          <t>https://leetcode.com/problems/longest-consecutive-sequence/</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1500,7 +1479,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1510,17 +1489,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>HashMap / HashSet</t>
+          <t>Intervals</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Sequence</t>
+          <t>Sorting + Merge</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Longest Consecutive Sequence</t>
+          <t>Merge Intervals</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1535,12 +1514,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/longest-consecutive-sequence/</t>
+          <t>https://leetcode.com/problems/merge-intervals/</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1550,7 +1529,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1560,22 +1539,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Intervals</t>
+          <t>Sorting</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Sorting + Merge</t>
+          <t>Custom Sort</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Merge Intervals</t>
+          <t>Sort an Array</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy-Medium</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1585,12 +1564,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/merge-intervals/</t>
+          <t>https://leetcode.com/problems/sort-an-array/</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1600,7 +1579,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1615,17 +1594,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Custom Sort</t>
+          <t>Kth Element</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Sort an Array</t>
+          <t>Kth Largest Element in an Array</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Easy-Medium</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1635,7 +1614,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/sort-an-array/</t>
+          <t>https://leetcode.com/problems/kth-largest-element-in-an-array/</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1660,22 +1639,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Sorting</t>
+          <t>Intervals</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Kth Element</t>
+          <t>Overlap Check</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Kth Largest Element in an Array</t>
+          <t>Meeting Rooms</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1685,7 +1664,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/kth-largest-element-in-an-array/</t>
+          <t>https://leetcode.com/problems/meeting-rooms/</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1710,17 +1689,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Intervals</t>
+          <t>Binary Search</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Overlap Check</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Meeting Rooms</t>
+          <t>Binary Search</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1735,12 +1714,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/meeting-rooms/</t>
+          <t>https://leetcode.com/problems/binary-search/</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1750,7 +1729,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1765,12 +1744,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Insert Position</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Binary Search</t>
+          <t>Search Insert Position</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1785,7 +1764,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/binary-search/</t>
+          <t>https://leetcode.com/problems/search-insert-position/</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1815,12 +1794,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Insert Position</t>
+          <t>Boundary Search</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Search Insert Position</t>
+          <t>First Bad Version</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1835,12 +1814,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/search-insert-position/</t>
+          <t>https://leetcode.com/problems/first-bad-version/</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1850,7 +1829,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1865,17 +1844,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Boundary Search</t>
+          <t>Rotated Array</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>First Bad Version</t>
+          <t>Search in Rotated Sorted Array</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1885,7 +1864,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/first-bad-version/</t>
+          <t>https://leetcode.com/problems/search-in-rotated-sorted-array/</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1915,12 +1894,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Rotated Array</t>
+          <t>Range Search</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Search in Rotated Sorted Array</t>
+          <t>Find First and Last Position of Element in Sorted Array</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1935,7 +1914,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/search-in-rotated-sorted-array/</t>
+          <t>https://leetcode.com/problems/find-first-and-last-position-of-element-in-sorted-array/</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1960,17 +1939,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Binary Search</t>
+          <t>Two Pointers</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Range Search</t>
+          <t>Sum</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Find First and Last Position of Element in Sorted Array</t>
+          <t>3Sum</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1985,7 +1964,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/find-first-and-last-position-of-element-in-sorted-array/</t>
+          <t>https://leetcode.com/problems/3sum/</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2015,12 +1994,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Sum</t>
+          <t>Container</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>3Sum</t>
+          <t>Container With Most Water</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2035,7 +2014,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/3sum/</t>
+          <t>https://leetcode.com/problems/container-with-most-water/</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -2065,17 +2044,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Container</t>
+          <t>Removal</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Container With Most Water</t>
+          <t>Remove Duplicates from Sorted Array</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2085,12 +2064,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/container-with-most-water/</t>
+          <t>https://leetcode.com/problems/remove-duplicates-from-sorted-array/</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2100,7 +2079,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2110,17 +2089,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Two Pointers</t>
+          <t>Number Theory</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Removal</t>
+          <t>LCM</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Remove Duplicates from Sorted Array</t>
+          <t>LCM of Two Numbers</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2130,12 +2109,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/remove-duplicates-from-sorted-array/</t>
+          <t>https://www.geeksforgeeks.org/program-to-find-lcm-of-two-numbers/</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2160,17 +2139,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Number Theory</t>
+          <t>Sliding Window</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>LCM</t>
+          <t>Fixed Window</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>LCM of Two Numbers</t>
+          <t>Maximum Average Subarray I</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2180,17 +2159,17 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/program-to-find-lcm-of-two-numbers/</t>
+          <t>https://leetcode.com/problems/maximum-average-subarray-i/</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2200,7 +2179,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2215,17 +2194,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Fixed Window</t>
+          <t>Variable Window</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Maximum Average Subarray I</t>
+          <t>Minimum Size Subarray Sum</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2235,12 +2214,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/maximum-average-subarray-i/</t>
+          <t>https://leetcode.com/problems/minimum-size-subarray-sum/</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2250,7 +2229,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2265,12 +2244,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Variable Window</t>
+          <t>Char Frequency</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Minimum Size Subarray Sum</t>
+          <t>Permutation in String</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2285,12 +2264,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/minimum-size-subarray-sum/</t>
+          <t>https://leetcode.com/problems/permutation-in-string/</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2300,7 +2279,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2310,22 +2289,22 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Sliding Window</t>
+          <t>Prefix Sum</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Char Frequency</t>
+          <t>Range Sum</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Permutation in String</t>
+          <t>Range Sum Query - Immutable</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2335,7 +2314,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/permutation-in-string/</t>
+          <t>https://leetcode.com/problems/range-sum-query-immutable/</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2365,12 +2344,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Range Sum</t>
+          <t>Equilibrium Point</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Range Sum Query - Immutable</t>
+          <t>Find Pivot Index</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2385,7 +2364,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/range-sum-query-immutable/</t>
+          <t>https://leetcode.com/problems/find-pivot-index/</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2410,22 +2389,22 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Prefix Sum</t>
+          <t>Matrix</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Equilibrium Point</t>
+          <t>Traversal</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Find Pivot Index</t>
+          <t>Spiral Matrix</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2435,12 +2414,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/find-pivot-index/</t>
+          <t>https://leetcode.com/problems/spiral-matrix/</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2450,7 +2429,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2465,12 +2444,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Traversal</t>
+          <t>Rotation</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Spiral Matrix</t>
+          <t>Rotate Image</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2485,12 +2464,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/spiral-matrix/</t>
+          <t>https://leetcode.com/problems/rotate-image/</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2500,7 +2479,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2515,12 +2494,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Rotation</t>
+          <t>Search</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Rotate Image</t>
+          <t>Search a 2D Matrix</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2535,7 +2514,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/rotate-image/</t>
+          <t>https://leetcode.com/problems/search-a-2d-matrix/</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2565,12 +2544,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Search</t>
+          <t>Modification</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Search a 2D Matrix</t>
+          <t>Set Matrix Zeroes</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2585,7 +2564,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/search-a-2d-matrix/</t>
+          <t>https://leetcode.com/problems/set-matrix-zeroes/</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2610,22 +2589,22 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Matrix</t>
+          <t>Recursion</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Modification</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Set Matrix Zeroes</t>
+          <t>Fibonacci Number</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2635,12 +2614,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/set-matrix-zeroes/</t>
+          <t>https://leetcode.com/problems/fibonacci-number/</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2650,7 +2629,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2665,17 +2644,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Power/Exponent</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Fibonacci Number</t>
+          <t>Pow(x, n)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2685,12 +2664,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/fibonacci-number/</t>
+          <t>https://leetcode.com/problems/powx-n/</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2700,7 +2679,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -2710,22 +2689,22 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Recursion</t>
+          <t>Mathematics</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Power/Exponent</t>
+          <t>Digit Sum</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Pow(x, n)</t>
+          <t>Add Digits</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2735,7 +2714,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/powx-n/</t>
+          <t>https://leetcode.com/problems/add-digits/</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2750,7 +2729,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2760,22 +2739,22 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Mathematics</t>
+          <t>Basic Backtracking</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Digit Sum</t>
+          <t>Subsets</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Add Digits</t>
+          <t>Subsets</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2785,7 +2764,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/add-digits/</t>
+          <t>https://leetcode.com/problems/subsets/</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2815,12 +2794,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Subsets</t>
+          <t>Permutations</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Subsets</t>
+          <t>Permutations</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2835,7 +2814,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/subsets/</t>
+          <t>https://leetcode.com/problems/permutations/</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2865,12 +2844,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Permutations</t>
+          <t>Combination</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Permutations</t>
+          <t>Combination Sum</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2885,7 +2864,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/permutations/</t>
+          <t>https://leetcode.com/problems/combination-sum/</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2910,22 +2889,22 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Basic Backtracking</t>
+          <t>Stack</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Combination</t>
+          <t>Validity Check</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Combination Sum</t>
+          <t>Valid Parentheses</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2935,12 +2914,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/combination-sum/</t>
+          <t>https://leetcode.com/problems/valid-parentheses/</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2950,7 +2929,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2965,17 +2944,17 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Validity Check</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Valid Parentheses</t>
+          <t>Min Stack</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2985,7 +2964,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/valid-parentheses/</t>
+          <t>https://leetcode.com/problems/min-stack/</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -3015,12 +2994,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Evaluation</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Min Stack</t>
+          <t>Evaluate Reverse Polish Notation</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -3035,12 +3014,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/min-stack/</t>
+          <t>https://leetcode.com/problems/evaluate-reverse-polish-notation/</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3050,7 +3029,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3065,12 +3044,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Evaluation</t>
+          <t>Monotonic Stack</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Evaluate Reverse Polish Notation</t>
+          <t>Daily Temperatures</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -3085,7 +3064,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/evaluate-reverse-polish-notation/</t>
+          <t>https://leetcode.com/problems/daily-temperatures/</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -3115,12 +3094,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Monotonic Stack</t>
+          <t>Path Simplification</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Daily Temperatures</t>
+          <t>Simplify Path</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -3135,7 +3114,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/daily-temperatures/</t>
+          <t>https://leetcode.com/problems/simplify-path/</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -3150,7 +3129,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3160,22 +3139,22 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Stack</t>
+          <t>Queue</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Path Simplification</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Simplify Path</t>
+          <t>Implement Queue using Stacks</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -3185,7 +3164,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/simplify-path/</t>
+          <t>https://leetcode.com/problems/implement-queue-using-stacks/</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -3200,7 +3179,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3210,37 +3189,37 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Queue</t>
+          <t>Number Theory</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Prime Factorization</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Implement Queue using Stacks</t>
+          <t>Prime Factors of a Number</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Easy-Medium</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/implement-queue-using-stacks/</t>
+          <t>https://www.geeksforgeeks.org/prime-factor/</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3250,7 +3229,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3260,37 +3239,37 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Number Theory</t>
+          <t>Queue</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Prime Factorization</t>
+          <t>Sliding Window</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Prime Factors of a Number</t>
+          <t>Sliding Window Maximum</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Easy-Medium</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/prime-factor/</t>
+          <t>https://leetcode.com/problems/sliding-window-maximum/</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3300,7 +3279,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3310,22 +3289,22 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Queue</t>
+          <t>Linked List</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Sliding Window</t>
+          <t>Reversal</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Sliding Window Maximum</t>
+          <t>Reverse Linked List</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -3335,12 +3314,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/sliding-window-maximum/</t>
+          <t>https://leetcode.com/problems/reverse-linked-list/</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3350,7 +3329,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3365,12 +3344,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Reversal</t>
+          <t>Two Pointer</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Reverse Linked List</t>
+          <t>Middle of the Linked List</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -3385,7 +3364,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/reverse-linked-list/</t>
+          <t>https://leetcode.com/problems/middle-of-the-linked-list/</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -3415,12 +3394,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Two Pointer</t>
+          <t>Cycle Detection</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Middle of the Linked List</t>
+          <t>Linked List Cycle</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -3435,7 +3414,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/middle-of-the-linked-list/</t>
+          <t>https://leetcode.com/problems/linked-list-cycle/</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -3465,12 +3444,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Cycle Detection</t>
+          <t>Merge</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Linked List Cycle</t>
+          <t>Merge Two Sorted Lists</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3485,7 +3464,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/linked-list-cycle/</t>
+          <t>https://leetcode.com/problems/merge-two-sorted-lists/</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -3515,17 +3494,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Merge</t>
+          <t>Removal</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Merge Two Sorted Lists</t>
+          <t>Remove Nth Node From End of List</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -3535,12 +3514,12 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/merge-two-sorted-lists/</t>
+          <t>https://leetcode.com/problems/remove-nth-node-from-end-of-list/</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -3550,7 +3529,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3565,17 +3544,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Removal</t>
+          <t>Palindrome Check</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Remove Nth Node From End of List</t>
+          <t>Palindrome Linked List</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3585,7 +3564,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/remove-nth-node-from-end-of-list/</t>
+          <t>https://leetcode.com/problems/palindrome-linked-list/</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -3615,12 +3594,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Palindrome Check</t>
+          <t>Intersection</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Palindrome Linked List</t>
+          <t>Intersection of Two Linked Lists</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3635,7 +3614,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/palindrome-linked-list/</t>
+          <t>https://leetcode.com/problems/intersection-of-two-linked-lists/</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -3660,17 +3639,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Linked List</t>
+          <t>Trees</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Intersection</t>
+          <t>Traversal</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Intersection of Two Linked Lists</t>
+          <t>Maximum Depth of Binary Tree</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3685,12 +3664,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/intersection-of-two-linked-lists/</t>
+          <t>https://leetcode.com/problems/maximum-depth-of-binary-tree/</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -3700,7 +3679,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3715,17 +3694,17 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Traversal</t>
+          <t>BFS</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Maximum Depth of Binary Tree</t>
+          <t>Binary Tree Level Order Traversal</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -3735,7 +3714,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/maximum-depth-of-binary-tree/</t>
+          <t>https://leetcode.com/problems/binary-tree-level-order-traversal/</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -3765,17 +3744,17 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>BFS</t>
+          <t>Diameter</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Binary Tree Level Order Traversal</t>
+          <t>Diameter of Binary Tree</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy-Medium</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3785,12 +3764,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/binary-tree-level-order-traversal/</t>
+          <t>https://leetcode.com/problems/diameter-of-binary-tree/</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -3800,7 +3779,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3815,17 +3794,17 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Diameter</t>
+          <t>Recursion</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Diameter of Binary Tree</t>
+          <t>Invert Binary Tree</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Easy-Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3835,7 +3814,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/diameter-of-binary-tree/</t>
+          <t>https://leetcode.com/problems/invert-binary-tree/</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -3865,12 +3844,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Recursion</t>
+          <t>Symmetry Check</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Invert Binary Tree</t>
+          <t>Symmetric Tree</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3885,7 +3864,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/invert-binary-tree/</t>
+          <t>https://leetcode.com/problems/symmetric-tree/</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3915,12 +3894,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Symmetry Check</t>
+          <t>Path Sum</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Symmetric Tree</t>
+          <t>Path Sum</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3935,7 +3914,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/symmetric-tree/</t>
+          <t>https://leetcode.com/problems/path-sum/</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -3960,22 +3939,22 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Trees</t>
+          <t>Binary Search Trees</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Path Sum</t>
+          <t>Validation</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Path Sum</t>
+          <t>Validate Binary Search Tree</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3985,7 +3964,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/path-sum/</t>
+          <t>https://leetcode.com/problems/validate-binary-search-tree/</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -4015,17 +3994,17 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Validation</t>
+          <t>Lowest Common Ancestor</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Validate Binary Search Tree</t>
+          <t>Lowest Common Ancestor of a Binary Search Tree</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy-Medium</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -4035,7 +4014,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/validate-binary-search-tree/</t>
+          <t>https://leetcode.com/problems/lowest-common-ancestor-of-a-binary-search-tree/</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -4060,37 +4039,37 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Binary Search Trees</t>
+          <t>Pattern-based Logic</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Lowest Common Ancestor</t>
+          <t>Pattern Printing</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Lowest Common Ancestor of a Binary Search Tree</t>
+          <t>Star / Number Pattern Printing</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Easy-Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/lowest-common-ancestor-of-a-binary-search-tree/</t>
+          <t>https://www.geeksforgeeks.org/printing-patterns-using-loops/</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -4100,7 +4079,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -4110,17 +4089,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Pattern-based Logic</t>
+          <t>Heap / Priority Queue</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Pattern Printing</t>
+          <t>Kth Largest</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Star / Number Pattern Printing</t>
+          <t>Kth Largest Element in a Stream</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -4130,17 +4109,17 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/printing-patterns-using-loops/</t>
+          <t>https://leetcode.com/problems/kth-largest-element-in-a-stream/</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -4150,7 +4129,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -4165,17 +4144,17 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Kth Largest</t>
+          <t>Merge</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Kth Largest Element in a Stream</t>
+          <t>Merge k Sorted Lists</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -4185,7 +4164,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/kth-largest-element-in-a-stream/</t>
+          <t>https://leetcode.com/problems/merge-k-sorted-lists/</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -4200,7 +4179,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -4215,12 +4194,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Merge</t>
+          <t>Top K</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Merge k Sorted Lists</t>
+          <t>Top K Frequent Words</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -4235,7 +4214,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/merge-k-sorted-lists/</t>
+          <t>https://leetcode.com/problems/top-k-frequent-words/</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -4250,7 +4229,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -4260,17 +4239,17 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Heap / Priority Queue</t>
+          <t>Greedy Algorithms</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Top K</t>
+          <t>Jump Game</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Top K Frequent Words</t>
+          <t>Jump Game</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -4285,7 +4264,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/top-k-frequent-words/</t>
+          <t>https://leetcode.com/problems/jump-game/</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -4315,12 +4294,12 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Jump Game</t>
+          <t>Interval Scheduling</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Jump Game</t>
+          <t>Non-overlapping Intervals</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -4335,7 +4314,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/jump-game/</t>
+          <t>https://leetcode.com/problems/non-overlapping-intervals/</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -4360,22 +4339,22 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Greedy Algorithms</t>
+          <t>Simulation</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Interval Scheduling</t>
+          <t>Grid Simulation</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Non-overlapping Intervals</t>
+          <t>Robot Return to Origin</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -4385,7 +4364,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/non-overlapping-intervals/</t>
+          <t>https://leetcode.com/problems/robot-return-to-origin/</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -4410,17 +4389,17 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Simulation</t>
+          <t>Dynamic Programming</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Grid Simulation</t>
+          <t>1D DP</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Robot Return to Origin</t>
+          <t>Climbing Stairs</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -4435,12 +4414,12 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/robot-return-to-origin/</t>
+          <t>https://leetcode.com/problems/climbing-stairs/</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -4450,7 +4429,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -4470,12 +4449,12 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Climbing Stairs</t>
+          <t>House Robber</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -4485,7 +4464,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/climbing-stairs/</t>
+          <t>https://leetcode.com/problems/house-robber/</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -4515,12 +4494,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>1D DP</t>
+          <t>Coin Change</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>House Robber</t>
+          <t>Coin Change</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -4535,12 +4514,12 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/house-robber/</t>
+          <t>https://leetcode.com/problems/coin-change/</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -4550,7 +4529,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -4565,12 +4544,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Coin Change</t>
+          <t>Subsequence</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Coin Change</t>
+          <t>Longest Increasing Subsequence</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -4585,7 +4564,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/coin-change/</t>
+          <t>https://leetcode.com/problems/longest-increasing-subsequence/</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -4615,12 +4594,12 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Subsequence</t>
+          <t>Grid DP</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Longest Increasing Subsequence</t>
+          <t>Unique Paths</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -4635,7 +4614,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/longest-increasing-subsequence/</t>
+          <t>https://leetcode.com/problems/unique-paths/</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -4660,22 +4639,22 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Dynamic Programming</t>
+          <t>Graph Basics</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Grid DP</t>
+          <t>Flood Fill</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Unique Paths</t>
+          <t>Flood Fill</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -4685,12 +4664,12 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/unique-paths/</t>
+          <t>https://leetcode.com/problems/flood-fill/</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -4700,7 +4679,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -4715,17 +4694,17 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Flood Fill</t>
+          <t>Islands / DFS</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Flood Fill</t>
+          <t>Number of Islands</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -4735,7 +4714,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/flood-fill/</t>
+          <t>https://leetcode.com/problems/number-of-islands/</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -4765,12 +4744,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Islands / DFS</t>
+          <t>BFS</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Number of Islands</t>
+          <t>Rotting Oranges</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -4785,12 +4764,12 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/number-of-islands/</t>
+          <t>https://leetcode.com/problems/rotting-oranges/</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -4800,7 +4779,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -4815,12 +4794,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>BFS</t>
+          <t>DFS</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Rotting Oranges</t>
+          <t>Clone Graph</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4835,7 +4814,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/rotting-oranges/</t>
+          <t>https://leetcode.com/problems/clone-graph/</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -4850,7 +4829,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -4860,22 +4839,22 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Graph Basics</t>
+          <t>Mathematics</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>DFS</t>
+          <t>Number Reversal</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Clone Graph</t>
+          <t>Palindrome Number</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -4885,12 +4864,12 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/clone-graph/</t>
+          <t>https://leetcode.com/problems/palindrome-number/</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -4900,7 +4879,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -4910,17 +4889,17 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Mathematics</t>
+          <t>Bit Manipulation</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Number Reversal</t>
+          <t>Bit Counting DP</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Palindrome Number</t>
+          <t>Counting Bits</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4935,12 +4914,12 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/palindrome-number/</t>
+          <t>https://leetcode.com/problems/counting-bits/</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -4950,7 +4929,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -4960,22 +4939,22 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Bit Manipulation</t>
+          <t>Number Theory</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Bit Counting DP</t>
+          <t>Sieve of Eratosthenes</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Counting Bits</t>
+          <t>Count Primes</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -4985,12 +4964,12 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/counting-bits/</t>
+          <t>https://leetcode.com/problems/count-primes/</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -5000,7 +4979,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -5010,22 +4989,22 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Number Theory</t>
+          <t>Miscellaneous</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Sieve of Eratosthenes</t>
+          <t>String Math</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Count Primes</t>
+          <t>Greatest Common Divisor of Strings</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -5035,12 +5014,12 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/count-primes/</t>
+          <t>https://leetcode.com/problems/greatest-common-divisor-of-strings/</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -5050,60 +5029,11 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="15.75" customHeight="1">
-      <c r="A92" t="n">
-        <v>91</v>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>Miscellaneous</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>String Math</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>Greatest Common Divisor of Strings</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>LeetCode</t>
-        </is>
-      </c>
-      <c r="G92" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/problems/greatest-common-divisor-of-strings/</t>
-        </is>
-      </c>
-      <c r="H92" t="inlineStr">
-        <is>
-          <t>Similar</t>
-        </is>
-      </c>
-      <c r="I92" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J92" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="15.75" customHeight="1"/>
     <row r="93" ht="15.75" customHeight="1"/>
     <row r="94" ht="15.75" customHeight="1"/>
     <row r="95" ht="15.75" customHeight="1"/>
@@ -6042,7 +5972,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Topic-wise Question Distribution</t>
         </is>
@@ -6066,405 +5996,405 @@
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Arrays</t>
         </is>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B4)</f>
         <v/>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B5)</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Strings</t>
         </is>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B6)</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Number Theory</t>
         </is>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B7)</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Frequency Counting</t>
         </is>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B8)</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>HashMap / HashSet</t>
         </is>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B9)</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Intervals</t>
         </is>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B10)</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Sorting</t>
         </is>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B11)</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Binary Search</t>
         </is>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B12)</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Two Pointers</t>
         </is>
       </c>
-      <c r="C13" s="2">
+      <c r="C13" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B13)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Sliding Window</t>
         </is>
       </c>
-      <c r="C14" s="2">
+      <c r="C14" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B14)</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Prefix Sum</t>
         </is>
       </c>
-      <c r="C15" s="2">
+      <c r="C15" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B15)</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Matrix</t>
         </is>
       </c>
-      <c r="C16" s="2">
+      <c r="C16" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B16)</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="2" t="n">
+      <c r="A17" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Recursion</t>
         </is>
       </c>
-      <c r="C17" s="2">
+      <c r="C17" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B17)</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="2" t="n">
+      <c r="A18" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Basic Backtracking</t>
         </is>
       </c>
-      <c r="C18" s="2">
+      <c r="C18" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B18)</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
-      <c r="A19" s="2" t="n">
+      <c r="A19" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Stack</t>
         </is>
       </c>
-      <c r="C19" s="2">
+      <c r="C19" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B19)</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>Queue</t>
         </is>
       </c>
-      <c r="C20" s="2">
+      <c r="C20" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B20)</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Linked List</t>
         </is>
       </c>
-      <c r="C21" s="2">
+      <c r="C21" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B21)</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="2" t="n">
+      <c r="A22" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>Trees</t>
         </is>
       </c>
-      <c r="C22" s="2">
+      <c r="C22" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B22)</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="2" t="n">
+      <c r="A23" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>Binary Search Trees</t>
         </is>
       </c>
-      <c r="C23" s="2">
+      <c r="C23" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B23)</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="2" t="n">
+      <c r="A24" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>Pattern-based Logic</t>
         </is>
       </c>
-      <c r="C24" s="2">
+      <c r="C24" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B24)</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="2" t="n">
+      <c r="A25" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>Heap / Priority Queue</t>
         </is>
       </c>
-      <c r="C25" s="2">
+      <c r="C25" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B25)</f>
         <v/>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="2" t="n">
+      <c r="A26" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>Greedy Algorithms</t>
         </is>
       </c>
-      <c r="C26" s="2">
+      <c r="C26" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B26)</f>
         <v/>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="2" t="n">
+      <c r="A27" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>Simulation</t>
         </is>
       </c>
-      <c r="C27" s="2">
+      <c r="C27" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B27)</f>
         <v/>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="2" t="n">
+      <c r="A28" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>Dynamic Programming</t>
         </is>
       </c>
-      <c r="C28" s="2">
+      <c r="C28" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B28)</f>
         <v/>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="2" t="n">
+      <c r="A29" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>Graph Basics</t>
         </is>
       </c>
-      <c r="C29" s="2">
+      <c r="C29" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B29)</f>
         <v/>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="2" t="n">
+      <c r="A30" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>Bit Manipulation</t>
         </is>
       </c>
-      <c r="C30" s="2">
+      <c r="C30" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B30)</f>
         <v/>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="2" t="n">
+      <c r="A31" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>Miscellaneous</t>
         </is>
       </c>
-      <c r="C31" s="2">
+      <c r="C31" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$B$2:$B$101,B31)</f>
         <v/>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="12" t="n"/>
-      <c r="B32" s="13" t="inlineStr">
+      <c r="A32" s="5" t="n"/>
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C32" s="13">
+      <c r="C32" s="6">
         <f>SUM(C4:C31)</f>
         <v/>
       </c>
@@ -7469,7 +7399,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Difficulty Distribution</t>
         </is>
@@ -7493,55 +7423,55 @@
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Easy</t>
         </is>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$E$2:$E$101,B4)</f>
         <v/>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Easy-Medium</t>
         </is>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$E$2:$E$101,B5)</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="C6" s="2">
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C6" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!$E$2:$E$101,B6)</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="12" t="n"/>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="A7" s="5" t="n"/>
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C7" s="13">
+      <c r="C7" s="6">
         <f>SUM(C4:C6)</f>
         <v/>
       </c>
@@ -8558,7 +8488,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Deloitte Prep — Progress Tracker</t>
         </is>
@@ -8577,105 +8507,105 @@
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Total Questions</t>
         </is>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="3">
         <f>COUNTA('Master Sheet (100 Qs)'!A2:A101)</f>
         <v/>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Solved (Status = Done)</t>
         </is>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!K2:K101,"Done")</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>In Progress (Status = In Progress)</t>
         </is>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!K2:K101,"In Progress")</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="3">
         <f>COUNTA('Master Sheet (100 Qs)'!A2:A101)-COUNTIF('Master Sheet (100 Qs)'!K2:K101,"Done")-COUNTIF('Master Sheet (100 Qs)'!K2:K101,"In Progress")</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Completion %</t>
         </is>
       </c>
-      <c r="B8" s="2">
+      <c r="B8" s="3">
         <f>ROUND(COUNTIF('Master Sheet (100 Qs)'!K2:K101,"Done")/COUNTA('Master Sheet (100 Qs)'!A2:A101)*100,1)</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>High Importance Solved</t>
         </is>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" s="3">
         <f>_xlfn.COUNTIFS('Master Sheet (100 Qs)'!J2:J101,"High",'Master Sheet (100 Qs)'!K2:K101,"Done")</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Total High Importance Qs</t>
         </is>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="3">
         <f>COUNTIF('Master Sheet (100 Qs)'!J2:J101,"High")</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
-      <c r="A13" s="17" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>Instructions:</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>1. Go to 'Master Sheet (100 Qs)', column K (Status).</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="17" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>2. Type 'Done', 'In Progress', or leave blank for each question as you practice.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="17" t="inlineStr">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>3. This tracker updates automatically using formulas.</t>
         </is>

</xml_diff>

<commit_message>
feat: Unique Paths added — pid 70, sheet updated
</commit_message>
<xml_diff>
--- a/Sheets/Deloitte_100_Coding_Questions.xlsx
+++ b/Sheets/Deloitte_100_Coding_Questions.xlsx
@@ -544,17 +544,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Kadane's Algorithm</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Maximum Subarray</t>
+          <t>Contains Duplicate</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Easy-Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -564,7 +564,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/maximum-subarray/</t>
+          <t>https://leetcode.com/problems/contains-duplicate/</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -594,17 +594,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Prefix Product</t>
+          <t>Kadane's Algorithm</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Product of Array Except Self</t>
+          <t>Maximum Subarray</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy-Medium</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -614,12 +614,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/product-of-array-except-self/</t>
+          <t>https://leetcode.com/problems/maximum-subarray/</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -644,17 +644,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Merging</t>
+          <t>Prefix Product</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Merge Sorted Array</t>
+          <t>Product of Array Except Self</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -664,7 +664,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/merge-sorted-array/</t>
+          <t>https://leetcode.com/problems/product-of-array-except-self/</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -694,12 +694,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Missing Element</t>
+          <t>Merging</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Missing Number</t>
+          <t>Merge Sorted Array</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -714,12 +714,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/missing-number/</t>
+          <t>https://leetcode.com/problems/merge-sorted-array/</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -729,7 +729,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -739,17 +739,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Mathematics</t>
+          <t>Arrays</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Digit Manipulation</t>
+          <t>Missing Element</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Armstrong Number</t>
+          <t>Missing Number</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -759,12 +759,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/c-program-to-check-armstrong-number/</t>
+          <t>https://leetcode.com/problems/missing-number/</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -789,17 +789,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Strings</t>
+          <t>Mathematics</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Anagram</t>
+          <t>Digit Manipulation</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Valid Anagram</t>
+          <t>Armstrong Number</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -809,12 +809,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/valid-anagram/</t>
+          <t>https://www.geeksforgeeks.org/c-program-to-check-armstrong-number/</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -844,12 +844,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Palindrome</t>
+          <t>Anagram</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Valid Palindrome</t>
+          <t>Valid Anagram</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/valid-palindrome/</t>
+          <t>https://leetcode.com/problems/valid-anagram/</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -894,17 +894,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Reversal</t>
+          <t>Palindrome</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Reverse Words in a String</t>
+          <t>Valid Palindrome</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -914,12 +914,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/reverse-words-in-a-string/</t>
+          <t>https://leetcode.com/problems/valid-palindrome/</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -944,12 +944,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Sliding Window</t>
+          <t>Reversal</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Longest Substring Without Repeating Characters</t>
+          <t>Reverse Words in a String</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -964,12 +964,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/longest-substring-without-repeating-characters/</t>
+          <t>https://leetcode.com/problems/reverse-words-in-a-string/</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -994,12 +994,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Compression</t>
+          <t>Sliding Window</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>String Compression</t>
+          <t>Longest Substring Without Repeating Characters</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1014,12 +1014,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/string-compression/</t>
+          <t>https://leetcode.com/problems/longest-substring-without-repeating-characters/</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1029,7 +1029,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1044,17 +1044,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Parsing</t>
+          <t>Compression</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Roman to Integer</t>
+          <t>String Compression</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/roman-to-integer/</t>
+          <t>https://leetcode.com/problems/string-compression/</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1089,17 +1089,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Number Theory</t>
+          <t>Strings</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>GCD</t>
+          <t>Parsing</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>GCD of Two Numbers (Euclidean Algorithm)</t>
+          <t>Roman to Integer</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1109,17 +1109,17 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/c-program-for-basic-euclidean-algorithms/</t>
+          <t>https://leetcode.com/problems/roman-to-integer/</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1129,7 +1129,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1139,37 +1139,37 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Strings</t>
+          <t>Number Theory</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Grouping</t>
+          <t>GCD</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Group Anagrams</t>
+          <t>GCD of Two Numbers (Euclidean Algorithm)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/group-anagrams/</t>
+          <t>https://www.geeksforgeeks.org/c-program-for-basic-euclidean-algorithms/</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1179,7 +1179,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1194,17 +1194,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Counting</t>
+          <t>Grouping</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>First Unique Character in a String</t>
+          <t>Group Anagrams</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/first-unique-character-in-a-string/</t>
+          <t>https://leetcode.com/problems/group-anagrams/</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1244,12 +1244,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Counting</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Longest Common Prefix</t>
+          <t>First Unique Character in a String</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/longest-common-prefix/</t>
+          <t>https://leetcode.com/problems/first-unique-character-in-a-string/</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1289,22 +1289,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>HashMap / HashSet</t>
+          <t>Strings</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Frequency</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Top K Frequent Elements</t>
+          <t>Longest Common Prefix</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1314,7 +1314,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/top-k-frequent-elements/</t>
+          <t>https://leetcode.com/problems/longest-common-prefix/</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1344,17 +1344,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Set Operations</t>
+          <t>Frequency</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Intersection of Two Arrays</t>
+          <t>Top K Frequent Elements</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1364,7 +1364,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/intersection-of-two-arrays/</t>
+          <t>https://leetcode.com/problems/top-k-frequent-elements/</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1394,42 +1394,42 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Subarray</t>
+          <t>Set Operations</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Subarray Sum Equals K</t>
+          <t>Intersection of Two Arrays</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>LeetCode</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/problems/intersection-of-two-arrays/</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Similar</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
           <t>Medium</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>LeetCode</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/problems/subarray-sum-equals-k/</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Community Report</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>High</t>
         </is>
       </c>
     </row>
@@ -1444,12 +1444,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Sequence</t>
+          <t>Subarray</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Longest Consecutive Sequence</t>
+          <t>Subarray Sum Equals K</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1464,12 +1464,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/longest-consecutive-sequence/</t>
+          <t>https://leetcode.com/problems/subarray-sum-equals-k/</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1479,7 +1479,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1489,17 +1489,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Intervals</t>
+          <t>HashMap / HashSet</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Sorting + Merge</t>
+          <t>Sequence</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Merge Intervals</t>
+          <t>Longest Consecutive Sequence</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1514,12 +1514,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/merge-intervals/</t>
+          <t>https://leetcode.com/problems/longest-consecutive-sequence/</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1529,7 +1529,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1539,22 +1539,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Sorting</t>
+          <t>Intervals</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Custom Sort</t>
+          <t>Sorting + Merge</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Sort an Array</t>
+          <t>Merge Intervals</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Easy-Medium</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1564,12 +1564,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/sort-an-array/</t>
+          <t>https://leetcode.com/problems/merge-intervals/</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1579,7 +1579,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1594,17 +1594,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Kth Element</t>
+          <t>Custom Sort</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Kth Largest Element in an Array</t>
+          <t>Sort an Array</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy-Medium</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/kth-largest-element-in-an-array/</t>
+          <t>https://leetcode.com/problems/sort-an-array/</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1639,22 +1639,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Intervals</t>
+          <t>Sorting</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Overlap Check</t>
+          <t>Kth Element</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Meeting Rooms</t>
+          <t>Kth Largest Element in an Array</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/meeting-rooms/</t>
+          <t>https://leetcode.com/problems/kth-largest-element-in-an-array/</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1689,17 +1689,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Binary Search</t>
+          <t>Intervals</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Overlap Check</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Binary Search</t>
+          <t>Meeting Rooms</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1714,12 +1714,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/binary-search/</t>
+          <t>https://leetcode.com/problems/meeting-rooms/</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1729,7 +1729,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1744,12 +1744,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Insert Position</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Search Insert Position</t>
+          <t>Binary Search</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/search-insert-position/</t>
+          <t>https://leetcode.com/problems/binary-search/</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1794,12 +1794,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Boundary Search</t>
+          <t>Insert Position</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>First Bad Version</t>
+          <t>Search Insert Position</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1814,12 +1814,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/first-bad-version/</t>
+          <t>https://leetcode.com/problems/search-insert-position/</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1829,7 +1829,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1844,17 +1844,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Rotated Array</t>
+          <t>Boundary Search</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Search in Rotated Sorted Array</t>
+          <t>First Bad Version</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/search-in-rotated-sorted-array/</t>
+          <t>https://leetcode.com/problems/first-bad-version/</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1894,12 +1894,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Range Search</t>
+          <t>Rotated Array</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Find First and Last Position of Element in Sorted Array</t>
+          <t>Search in Rotated Sorted Array</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/find-first-and-last-position-of-element-in-sorted-array/</t>
+          <t>https://leetcode.com/problems/search-in-rotated-sorted-array/</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1939,17 +1939,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Two Pointers</t>
+          <t>Binary Search</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Sum</t>
+          <t>Range Search</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>3Sum</t>
+          <t>Find First and Last Position of Element in Sorted Array</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/3sum/</t>
+          <t>https://leetcode.com/problems/find-first-and-last-position-of-element-in-sorted-array/</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1994,12 +1994,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Container</t>
+          <t>Sum</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Container With Most Water</t>
+          <t>3Sum</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2014,7 +2014,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/container-with-most-water/</t>
+          <t>https://leetcode.com/problems/3sum/</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -2044,17 +2044,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Removal</t>
+          <t>Container</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Remove Duplicates from Sorted Array</t>
+          <t>Container With Most Water</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2064,12 +2064,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/remove-duplicates-from-sorted-array/</t>
+          <t>https://leetcode.com/problems/container-with-most-water/</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2089,17 +2089,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Number Theory</t>
+          <t>Two Pointers</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>LCM</t>
+          <t>Removal</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>LCM of Two Numbers</t>
+          <t>Remove Duplicates from Sorted Array</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2109,12 +2109,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/program-to-find-lcm-of-two-numbers/</t>
+          <t>https://leetcode.com/problems/remove-duplicates-from-sorted-array/</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2139,17 +2139,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Sliding Window</t>
+          <t>Number Theory</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Fixed Window</t>
+          <t>LCM</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Maximum Average Subarray I</t>
+          <t>LCM of Two Numbers</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2159,17 +2159,17 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/maximum-average-subarray-i/</t>
+          <t>https://www.geeksforgeeks.org/program-to-find-lcm-of-two-numbers/</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2179,7 +2179,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2194,42 +2194,42 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Variable Window</t>
+          <t>Fixed Window</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Minimum Size Subarray Sum</t>
+          <t>Maximum Average Subarray I</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>LeetCode</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/problems/maximum-average-subarray-i/</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Similar</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
           <t>Medium</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>LeetCode</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/problems/minimum-size-subarray-sum/</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>Community Report</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>High</t>
         </is>
       </c>
     </row>
@@ -2244,12 +2244,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Char Frequency</t>
+          <t>Variable Window</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Permutation in String</t>
+          <t>Minimum Size Subarray Sum</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2264,12 +2264,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/permutation-in-string/</t>
+          <t>https://leetcode.com/problems/minimum-size-subarray-sum/</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2279,7 +2279,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2289,22 +2289,22 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Prefix Sum</t>
+          <t>Sliding Window</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Range Sum</t>
+          <t>Char Frequency</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Range Sum Query - Immutable</t>
+          <t>Permutation in String</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/range-sum-query-immutable/</t>
+          <t>https://leetcode.com/problems/permutation-in-string/</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2344,12 +2344,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Equilibrium Point</t>
+          <t>Range Sum</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Find Pivot Index</t>
+          <t>Range Sum Query - Immutable</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/find-pivot-index/</t>
+          <t>https://leetcode.com/problems/range-sum-query-immutable/</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2389,47 +2389,47 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Matrix</t>
+          <t>Prefix Sum</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Traversal</t>
+          <t>Equilibrium Point</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Spiral Matrix</t>
+          <t>Find Pivot Index</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>LeetCode</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/problems/find-pivot-index/</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Similar</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
           <t>Medium</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>LeetCode</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/problems/spiral-matrix/</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>Community Report</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>High</t>
         </is>
       </c>
     </row>
@@ -2444,12 +2444,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Rotation</t>
+          <t>Traversal</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Rotate Image</t>
+          <t>Spiral Matrix</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2464,12 +2464,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/rotate-image/</t>
+          <t>https://leetcode.com/problems/spiral-matrix/</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2479,7 +2479,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2494,12 +2494,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Search</t>
+          <t>Rotation</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Search a 2D Matrix</t>
+          <t>Rotate Image</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/search-a-2d-matrix/</t>
+          <t>https://leetcode.com/problems/rotate-image/</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2544,12 +2544,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Modification</t>
+          <t>Search</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Set Matrix Zeroes</t>
+          <t>Search a 2D Matrix</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/set-matrix-zeroes/</t>
+          <t>https://leetcode.com/problems/search-a-2d-matrix/</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2589,22 +2589,22 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Recursion</t>
+          <t>Matrix</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Modification</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Fibonacci Number</t>
+          <t>Set Matrix Zeroes</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2614,12 +2614,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/fibonacci-number/</t>
+          <t>https://leetcode.com/problems/set-matrix-zeroes/</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2644,17 +2644,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Power/Exponent</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Pow(x, n)</t>
+          <t>Fibonacci Number</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2664,12 +2664,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/powx-n/</t>
+          <t>https://leetcode.com/problems/fibonacci-number/</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2679,7 +2679,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2689,22 +2689,22 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Mathematics</t>
+          <t>Recursion</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Digit Sum</t>
+          <t>Power/Exponent</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Add Digits</t>
+          <t>Pow(x, n)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/add-digits/</t>
+          <t>https://leetcode.com/problems/powx-n/</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2729,7 +2729,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -2739,22 +2739,22 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Basic Backtracking</t>
+          <t>Mathematics</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Subsets</t>
+          <t>Digit Sum</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Subsets</t>
+          <t>Add Digits</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2764,7 +2764,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/subsets/</t>
+          <t>https://leetcode.com/problems/add-digits/</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2794,12 +2794,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Permutations</t>
+          <t>Subsets</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Permutations</t>
+          <t>Subsets</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2814,7 +2814,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/permutations/</t>
+          <t>https://leetcode.com/problems/subsets/</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2844,12 +2844,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Combination</t>
+          <t>Permutations</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Combination Sum</t>
+          <t>Permutations</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/combination-sum/</t>
+          <t>https://leetcode.com/problems/permutations/</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2889,22 +2889,22 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Stack</t>
+          <t>Basic Backtracking</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Validity Check</t>
+          <t>Combination</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Valid Parentheses</t>
+          <t>Combination Sum</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2914,12 +2914,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/valid-parentheses/</t>
+          <t>https://leetcode.com/problems/combination-sum/</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2944,17 +2944,17 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Validity Check</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Min Stack</t>
+          <t>Valid Parentheses</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2964,7 +2964,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/min-stack/</t>
+          <t>https://leetcode.com/problems/valid-parentheses/</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2994,12 +2994,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Evaluation</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Evaluate Reverse Polish Notation</t>
+          <t>Min Stack</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -3014,12 +3014,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/evaluate-reverse-polish-notation/</t>
+          <t>https://leetcode.com/problems/min-stack/</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3029,7 +3029,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3044,12 +3044,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Monotonic Stack</t>
+          <t>Evaluation</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Daily Temperatures</t>
+          <t>Evaluate Reverse Polish Notation</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/daily-temperatures/</t>
+          <t>https://leetcode.com/problems/evaluate-reverse-polish-notation/</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -3094,12 +3094,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Path Simplification</t>
+          <t>Monotonic Stack</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Simplify Path</t>
+          <t>Daily Temperatures</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/simplify-path/</t>
+          <t>https://leetcode.com/problems/daily-temperatures/</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -3129,7 +3129,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3139,22 +3139,22 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Queue</t>
+          <t>Stack</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Path Simplification</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Implement Queue using Stacks</t>
+          <t>Simplify Path</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -3164,7 +3164,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/implement-queue-using-stacks/</t>
+          <t>https://leetcode.com/problems/simplify-path/</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -3179,7 +3179,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3189,37 +3189,37 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Number Theory</t>
+          <t>Queue</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Prime Factorization</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Prime Factors of a Number</t>
+          <t>Implement Queue using Stacks</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Easy-Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/prime-factor/</t>
+          <t>https://leetcode.com/problems/implement-queue-using-stacks/</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3229,7 +3229,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3239,37 +3239,37 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Queue</t>
+          <t>Number Theory</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Sliding Window</t>
+          <t>Prime Factorization</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Sliding Window Maximum</t>
+          <t>Prime Factors of a Number</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy-Medium</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/sliding-window-maximum/</t>
+          <t>https://www.geeksforgeeks.org/prime-factor/</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3279,7 +3279,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3289,22 +3289,22 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Linked List</t>
+          <t>Queue</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Reversal</t>
+          <t>Sliding Window</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Reverse Linked List</t>
+          <t>Sliding Window Maximum</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -3314,12 +3314,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/reverse-linked-list/</t>
+          <t>https://leetcode.com/problems/sliding-window-maximum/</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3329,7 +3329,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3344,12 +3344,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Two Pointer</t>
+          <t>Reversal</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Middle of the Linked List</t>
+          <t>Reverse Linked List</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/middle-of-the-linked-list/</t>
+          <t>https://leetcode.com/problems/reverse-linked-list/</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -3394,12 +3394,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Cycle Detection</t>
+          <t>Two Pointer</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Linked List Cycle</t>
+          <t>Middle of the Linked List</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -3414,7 +3414,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/linked-list-cycle/</t>
+          <t>https://leetcode.com/problems/middle-of-the-linked-list/</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -3444,12 +3444,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Merge</t>
+          <t>Cycle Detection</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Merge Two Sorted Lists</t>
+          <t>Linked List Cycle</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3464,7 +3464,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/merge-two-sorted-lists/</t>
+          <t>https://leetcode.com/problems/linked-list-cycle/</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -3494,17 +3494,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Removal</t>
+          <t>Merge</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Remove Nth Node From End of List</t>
+          <t>Merge Two Sorted Lists</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -3514,12 +3514,12 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/remove-nth-node-from-end-of-list/</t>
+          <t>https://leetcode.com/problems/merge-two-sorted-lists/</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -3529,7 +3529,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3544,17 +3544,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Palindrome Check</t>
+          <t>Removal</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Palindrome Linked List</t>
+          <t>Remove Nth Node From End of List</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/palindrome-linked-list/</t>
+          <t>https://leetcode.com/problems/remove-nth-node-from-end-of-list/</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -3594,12 +3594,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Intersection</t>
+          <t>Palindrome Check</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Intersection of Two Linked Lists</t>
+          <t>Palindrome Linked List</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/intersection-of-two-linked-lists/</t>
+          <t>https://leetcode.com/problems/palindrome-linked-list/</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -3639,17 +3639,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Trees</t>
+          <t>Linked List</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Traversal</t>
+          <t>Intersection</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Maximum Depth of Binary Tree</t>
+          <t>Intersection of Two Linked Lists</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3664,12 +3664,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/maximum-depth-of-binary-tree/</t>
+          <t>https://leetcode.com/problems/intersection-of-two-linked-lists/</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3694,17 +3694,17 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>BFS</t>
+          <t>Traversal</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Binary Tree Level Order Traversal</t>
+          <t>Maximum Depth of Binary Tree</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/binary-tree-level-order-traversal/</t>
+          <t>https://leetcode.com/problems/maximum-depth-of-binary-tree/</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -3744,17 +3744,17 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Diameter</t>
+          <t>BFS</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Diameter of Binary Tree</t>
+          <t>Binary Tree Level Order Traversal</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Easy-Medium</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3764,12 +3764,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/diameter-of-binary-tree/</t>
+          <t>https://leetcode.com/problems/binary-tree-level-order-traversal/</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -3779,7 +3779,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3794,17 +3794,17 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Recursion</t>
+          <t>Diameter</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Invert Binary Tree</t>
+          <t>Diameter of Binary Tree</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Easy-Medium</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3814,7 +3814,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/invert-binary-tree/</t>
+          <t>https://leetcode.com/problems/diameter-of-binary-tree/</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -3844,12 +3844,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Symmetry Check</t>
+          <t>Recursion</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Symmetric Tree</t>
+          <t>Invert Binary Tree</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/symmetric-tree/</t>
+          <t>https://leetcode.com/problems/invert-binary-tree/</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3894,12 +3894,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Path Sum</t>
+          <t>Symmetry Check</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Path Sum</t>
+          <t>Symmetric Tree</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3914,7 +3914,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/path-sum/</t>
+          <t>https://leetcode.com/problems/symmetric-tree/</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -3939,22 +3939,22 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Binary Search Trees</t>
+          <t>Trees</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Validation</t>
+          <t>Path Sum</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Validate Binary Search Tree</t>
+          <t>Path Sum</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3964,7 +3964,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/validate-binary-search-tree/</t>
+          <t>https://leetcode.com/problems/path-sum/</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -3994,17 +3994,17 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Lowest Common Ancestor</t>
+          <t>Validation</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Lowest Common Ancestor of a Binary Search Tree</t>
+          <t>Validate Binary Search Tree</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Easy-Medium</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/lowest-common-ancestor-of-a-binary-search-tree/</t>
+          <t>https://leetcode.com/problems/validate-binary-search-tree/</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -4039,37 +4039,37 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Pattern-based Logic</t>
+          <t>Binary Search Trees</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Pattern Printing</t>
+          <t>Lowest Common Ancestor</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Star / Number Pattern Printing</t>
+          <t>Lowest Common Ancestor of a Binary Search Tree</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Easy-Medium</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/printing-patterns-using-loops/</t>
+          <t>https://leetcode.com/problems/lowest-common-ancestor-of-a-binary-search-tree/</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -4079,7 +4079,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -4089,17 +4089,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Heap / Priority Queue</t>
+          <t>Pattern-based Logic</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Kth Largest</t>
+          <t>Pattern Printing</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Kth Largest Element in a Stream</t>
+          <t>Star / Number Pattern Printing</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -4109,17 +4109,17 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/kth-largest-element-in-a-stream/</t>
+          <t>https://www.geeksforgeeks.org/printing-patterns-using-loops/</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -4129,7 +4129,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -4144,42 +4144,42 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Merge</t>
+          <t>Kth Largest</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Merge k Sorted Lists</t>
+          <t>Kth Largest Element in a Stream</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>LeetCode</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/problems/kth-largest-element-in-a-stream/</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Similar</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
           <t>Medium</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>LeetCode</t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/problems/merge-k-sorted-lists/</t>
-        </is>
-      </c>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>Similar</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>Low</t>
         </is>
       </c>
     </row>
@@ -4194,12 +4194,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Top K</t>
+          <t>Merge</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Top K Frequent Words</t>
+          <t>Merge k Sorted Lists</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/top-k-frequent-words/</t>
+          <t>https://leetcode.com/problems/merge-k-sorted-lists/</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -4229,7 +4229,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -4239,17 +4239,17 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Greedy Algorithms</t>
+          <t>Heap / Priority Queue</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Jump Game</t>
+          <t>Top K</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Jump Game</t>
+          <t>Top K Frequent Words</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/jump-game/</t>
+          <t>https://leetcode.com/problems/top-k-frequent-words/</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -4294,12 +4294,12 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Interval Scheduling</t>
+          <t>Jump Game</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Non-overlapping Intervals</t>
+          <t>Jump Game</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/non-overlapping-intervals/</t>
+          <t>https://leetcode.com/problems/jump-game/</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -4339,22 +4339,22 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Simulation</t>
+          <t>Greedy Algorithms</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Grid Simulation</t>
+          <t>Interval Scheduling</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Robot Return to Origin</t>
+          <t>Non-overlapping Intervals</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/robot-return-to-origin/</t>
+          <t>https://leetcode.com/problems/non-overlapping-intervals/</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -4389,17 +4389,17 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Dynamic Programming</t>
+          <t>Simulation</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>1D DP</t>
+          <t>Grid Simulation</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Climbing Stairs</t>
+          <t>Robot Return to Origin</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -4414,12 +4414,12 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/climbing-stairs/</t>
+          <t>https://leetcode.com/problems/robot-return-to-origin/</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -4429,7 +4429,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -4449,12 +4449,12 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>House Robber</t>
+          <t>Climbing Stairs</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/house-robber/</t>
+          <t>https://leetcode.com/problems/climbing-stairs/</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -4494,12 +4494,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Coin Change</t>
+          <t>1D DP</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Coin Change</t>
+          <t>House Robber</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -4514,12 +4514,12 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/coin-change/</t>
+          <t>https://leetcode.com/problems/house-robber/</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -4529,7 +4529,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -4544,12 +4544,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Subsequence</t>
+          <t>Coin Change</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Longest Increasing Subsequence</t>
+          <t>Coin Change</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -4564,7 +4564,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/longest-increasing-subsequence/</t>
+          <t>https://leetcode.com/problems/coin-change/</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -4594,12 +4594,12 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Grid DP</t>
+          <t>Subsequence</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Unique Paths</t>
+          <t>Longest Increasing Subsequence</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/unique-paths/</t>
+          <t>https://leetcode.com/problems/longest-increasing-subsequence/</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">

</xml_diff>

<commit_message>
cleanup: removed 4 more DB-existing problems from sheet (87 remaining)
</commit_message>
<xml_diff>
--- a/Sheets/Deloitte_100_Coding_Questions.xlsx
+++ b/Sheets/Deloitte_100_Coding_Questions.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K91"/>
+  <dimension ref="A1:K88"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.421875" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="6.00390625" customWidth="1" min="1" max="1"/>
@@ -544,12 +544,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Merging</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Contains Duplicate</t>
+          <t>Merge Sorted Array</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -564,12 +564,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/contains-duplicate/</t>
+          <t>https://leetcode.com/problems/merge-sorted-array/</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -579,7 +579,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -594,17 +594,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Kadane's Algorithm</t>
+          <t>Missing Element</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Maximum Subarray</t>
+          <t>Missing Number</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Easy-Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -614,7 +614,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/maximum-subarray/</t>
+          <t>https://leetcode.com/problems/missing-number/</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -639,37 +639,37 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Arrays</t>
+          <t>Mathematics</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Prefix Product</t>
+          <t>Digit Manipulation</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Product of Array Except Self</t>
+          <t>Armstrong Number</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/product-of-array-except-self/</t>
+          <t>https://www.geeksforgeeks.org/c-program-to-check-armstrong-number/</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -679,7 +679,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -689,17 +689,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Arrays</t>
+          <t>Strings</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Merging</t>
+          <t>Anagram</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Merge Sorted Array</t>
+          <t>Valid Anagram</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -714,12 +714,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/merge-sorted-array/</t>
+          <t>https://leetcode.com/problems/valid-anagram/</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -729,7 +729,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -739,17 +739,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Arrays</t>
+          <t>Strings</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Missing Element</t>
+          <t>Palindrome</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Missing Number</t>
+          <t>Valid Palindrome</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -764,7 +764,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/missing-number/</t>
+          <t>https://leetcode.com/problems/valid-palindrome/</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -789,37 +789,37 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Mathematics</t>
+          <t>Strings</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Digit Manipulation</t>
+          <t>Reversal</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Armstrong Number</t>
+          <t>Reverse Words in a String</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/c-program-to-check-armstrong-number/</t>
+          <t>https://leetcode.com/problems/reverse-words-in-a-string/</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -844,17 +844,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Anagram</t>
+          <t>Sliding Window</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Valid Anagram</t>
+          <t>Longest Substring Without Repeating Characters</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/valid-anagram/</t>
+          <t>https://leetcode.com/problems/longest-substring-without-repeating-characters/</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -894,17 +894,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Palindrome</t>
+          <t>Compression</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Valid Palindrome</t>
+          <t>String Compression</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -914,12 +914,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/valid-palindrome/</t>
+          <t>https://leetcode.com/problems/string-compression/</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -944,17 +944,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Reversal</t>
+          <t>Parsing</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Reverse Words in a String</t>
+          <t>Roman to Integer</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -964,7 +964,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/reverse-words-in-a-string/</t>
+          <t>https://leetcode.com/problems/roman-to-integer/</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -989,32 +989,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Strings</t>
+          <t>Number Theory</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Sliding Window</t>
+          <t>GCD</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Longest Substring Without Repeating Characters</t>
+          <t>GCD of Two Numbers (Euclidean Algorithm)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/longest-substring-without-repeating-characters/</t>
+          <t>https://www.geeksforgeeks.org/c-program-for-basic-euclidean-algorithms/</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1044,12 +1044,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Compression</t>
+          <t>Grouping</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>String Compression</t>
+          <t>Group Anagrams</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/string-compression/</t>
+          <t>https://leetcode.com/problems/group-anagrams/</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1094,12 +1094,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Parsing</t>
+          <t>Counting</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Roman to Integer</t>
+          <t>First Unique Character in a String</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/roman-to-integer/</t>
+          <t>https://leetcode.com/problems/first-unique-character-in-a-string/</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1139,17 +1139,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Number Theory</t>
+          <t>Strings</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>GCD</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>GCD of Two Numbers (Euclidean Algorithm)</t>
+          <t>Longest Common Prefix</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1159,17 +1159,17 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/c-program-for-basic-euclidean-algorithms/</t>
+          <t>https://leetcode.com/problems/longest-common-prefix/</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1179,7 +1179,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Strings</t>
+          <t>HashMap / HashSet</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Grouping</t>
+          <t>Frequency</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Group Anagrams</t>
+          <t>Top K Frequent Elements</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/group-anagrams/</t>
+          <t>https://leetcode.com/problems/top-k-frequent-elements/</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1239,17 +1239,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Strings</t>
+          <t>HashMap / HashSet</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Counting</t>
+          <t>Set Operations</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>First Unique Character in a String</t>
+          <t>Intersection of Two Arrays</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/first-unique-character-in-a-string/</t>
+          <t>https://leetcode.com/problems/intersection-of-two-arrays/</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1289,22 +1289,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Strings</t>
+          <t>HashMap / HashSet</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Subarray</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Longest Common Prefix</t>
+          <t>Subarray Sum Equals K</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1314,12 +1314,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/longest-common-prefix/</t>
+          <t>https://leetcode.com/problems/subarray-sum-equals-k/</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1329,7 +1329,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1344,12 +1344,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Frequency</t>
+          <t>Sequence</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Top K Frequent Elements</t>
+          <t>Longest Consecutive Sequence</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1364,7 +1364,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/top-k-frequent-elements/</t>
+          <t>https://leetcode.com/problems/longest-consecutive-sequence/</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1389,22 +1389,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>HashMap / HashSet</t>
+          <t>Intervals</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Set Operations</t>
+          <t>Sorting + Merge</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Intersection of Two Arrays</t>
+          <t>Merge Intervals</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1414,12 +1414,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/intersection-of-two-arrays/</t>
+          <t>https://leetcode.com/problems/merge-intervals/</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1439,47 +1439,47 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>HashMap / HashSet</t>
+          <t>Sorting</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Subarray</t>
+          <t>Custom Sort</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Subarray Sum Equals K</t>
+          <t>Sort an Array</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
+          <t>Easy-Medium</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>LeetCode</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/problems/sort-an-array/</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Similar</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
           <t>Medium</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>LeetCode</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/problems/subarray-sum-equals-k/</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Community Report</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>High</t>
         </is>
       </c>
     </row>
@@ -1489,17 +1489,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>HashMap / HashSet</t>
+          <t>Sorting</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Sequence</t>
+          <t>Kth Element</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Longest Consecutive Sequence</t>
+          <t>Kth Largest Element in an Array</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/longest-consecutive-sequence/</t>
+          <t>https://leetcode.com/problems/kth-largest-element-in-an-array/</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1544,42 +1544,42 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Sorting + Merge</t>
+          <t>Overlap Check</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Merge Intervals</t>
+          <t>Meeting Rooms</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>LeetCode</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/problems/meeting-rooms/</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Similar</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
           <t>Medium</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>LeetCode</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/problems/merge-intervals/</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>Community Report</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>High</t>
         </is>
       </c>
     </row>
@@ -1589,22 +1589,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Sorting</t>
+          <t>Binary Search</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Custom Sort</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Sort an Array</t>
+          <t>Binary Search</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Easy-Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1614,12 +1614,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/sort-an-array/</t>
+          <t>https://leetcode.com/problems/binary-search/</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1639,22 +1639,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Sorting</t>
+          <t>Binary Search</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Kth Element</t>
+          <t>Insert Position</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Kth Largest Element in an Array</t>
+          <t>Search Insert Position</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1664,12 +1664,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/kth-largest-element-in-an-array/</t>
+          <t>https://leetcode.com/problems/search-insert-position/</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1679,7 +1679,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1689,17 +1689,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Intervals</t>
+          <t>Binary Search</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Overlap Check</t>
+          <t>Boundary Search</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Meeting Rooms</t>
+          <t>First Bad Version</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/meeting-rooms/</t>
+          <t>https://leetcode.com/problems/first-bad-version/</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1744,17 +1744,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Rotated Array</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Binary Search</t>
+          <t>Search in Rotated Sorted Array</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1764,12 +1764,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/binary-search/</t>
+          <t>https://leetcode.com/problems/search-in-rotated-sorted-array/</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1794,17 +1794,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Insert Position</t>
+          <t>Range Search</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Search Insert Position</t>
+          <t>Find First and Last Position of Element in Sorted Array</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1814,12 +1814,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/search-insert-position/</t>
+          <t>https://leetcode.com/problems/find-first-and-last-position-of-element-in-sorted-array/</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1829,7 +1829,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1839,22 +1839,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Binary Search</t>
+          <t>Two Pointers</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Boundary Search</t>
+          <t>Sum</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>First Bad Version</t>
+          <t>3Sum</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/first-bad-version/</t>
+          <t>https://leetcode.com/problems/3sum/</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1889,17 +1889,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Binary Search</t>
+          <t>Two Pointers</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Rotated Array</t>
+          <t>Container</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Search in Rotated Sorted Array</t>
+          <t>Container With Most Water</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/search-in-rotated-sorted-array/</t>
+          <t>https://leetcode.com/problems/container-with-most-water/</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1939,22 +1939,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Binary Search</t>
+          <t>Two Pointers</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Range Search</t>
+          <t>Removal</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Find First and Last Position of Element in Sorted Array</t>
+          <t>Remove Duplicates from Sorted Array</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1964,12 +1964,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/find-first-and-last-position-of-element-in-sorted-array/</t>
+          <t>https://leetcode.com/problems/remove-duplicates-from-sorted-array/</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1979,7 +1979,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1989,37 +1989,37 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Two Pointers</t>
+          <t>Number Theory</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Sum</t>
+          <t>LCM</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>3Sum</t>
+          <t>LCM of Two Numbers</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/3sum/</t>
+          <t>https://www.geeksforgeeks.org/program-to-find-lcm-of-two-numbers/</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2029,7 +2029,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2039,22 +2039,22 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Two Pointers</t>
+          <t>Sliding Window</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Container</t>
+          <t>Fixed Window</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Container With Most Water</t>
+          <t>Maximum Average Subarray I</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/container-with-most-water/</t>
+          <t>https://leetcode.com/problems/maximum-average-subarray-i/</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2089,22 +2089,22 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Two Pointers</t>
+          <t>Sliding Window</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Removal</t>
+          <t>Variable Window</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Remove Duplicates from Sorted Array</t>
+          <t>Minimum Size Subarray Sum</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/remove-duplicates-from-sorted-array/</t>
+          <t>https://leetcode.com/problems/minimum-size-subarray-sum/</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2139,37 +2139,37 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Number Theory</t>
+          <t>Sliding Window</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>LCM</t>
+          <t>Char Frequency</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>LCM of Two Numbers</t>
+          <t>Permutation in String</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/program-to-find-lcm-of-two-numbers/</t>
+          <t>https://leetcode.com/problems/permutation-in-string/</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2179,7 +2179,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2189,17 +2189,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Sliding Window</t>
+          <t>Prefix Sum</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Fixed Window</t>
+          <t>Range Sum</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Maximum Average Subarray I</t>
+          <t>Range Sum Query - Immutable</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2214,7 +2214,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/maximum-average-subarray-i/</t>
+          <t>https://leetcode.com/problems/range-sum-query-immutable/</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2239,47 +2239,47 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Sliding Window</t>
+          <t>Prefix Sum</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Variable Window</t>
+          <t>Equilibrium Point</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Minimum Size Subarray Sum</t>
+          <t>Find Pivot Index</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>LeetCode</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/problems/find-pivot-index/</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Similar</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
           <t>Medium</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>LeetCode</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/problems/minimum-size-subarray-sum/</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>Community Report</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>High</t>
         </is>
       </c>
     </row>
@@ -2289,17 +2289,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Sliding Window</t>
+          <t>Matrix</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Char Frequency</t>
+          <t>Traversal</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Permutation in String</t>
+          <t>Spiral Matrix</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2314,12 +2314,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/permutation-in-string/</t>
+          <t>https://leetcode.com/problems/spiral-matrix/</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2339,22 +2339,22 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Prefix Sum</t>
+          <t>Matrix</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Range Sum</t>
+          <t>Rotation</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Range Sum Query - Immutable</t>
+          <t>Rotate Image</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/range-sum-query-immutable/</t>
+          <t>https://leetcode.com/problems/rotate-image/</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2389,22 +2389,22 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Prefix Sum</t>
+          <t>Matrix</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Equilibrium Point</t>
+          <t>Search</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Find Pivot Index</t>
+          <t>Search a 2D Matrix</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2414,7 +2414,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/find-pivot-index/</t>
+          <t>https://leetcode.com/problems/search-a-2d-matrix/</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2444,12 +2444,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Traversal</t>
+          <t>Modification</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Spiral Matrix</t>
+          <t>Set Matrix Zeroes</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2464,12 +2464,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/spiral-matrix/</t>
+          <t>https://leetcode.com/problems/set-matrix-zeroes/</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2479,7 +2479,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2489,22 +2489,22 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Matrix</t>
+          <t>Recursion</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Rotation</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Rotate Image</t>
+          <t>Fibonacci Number</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2514,12 +2514,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/rotate-image/</t>
+          <t>https://leetcode.com/problems/fibonacci-number/</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2539,17 +2539,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Matrix</t>
+          <t>Recursion</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Search</t>
+          <t>Power/Exponent</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Search a 2D Matrix</t>
+          <t>Pow(x, n)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/search-a-2d-matrix/</t>
+          <t>https://leetcode.com/problems/powx-n/</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2579,7 +2579,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -2589,22 +2589,22 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Matrix</t>
+          <t>Mathematics</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Modification</t>
+          <t>Digit Sum</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Set Matrix Zeroes</t>
+          <t>Add Digits</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/set-matrix-zeroes/</t>
+          <t>https://leetcode.com/problems/add-digits/</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2639,22 +2639,22 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Recursion</t>
+          <t>Basic Backtracking</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Subsets</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Fibonacci Number</t>
+          <t>Subsets</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2664,12 +2664,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/fibonacci-number/</t>
+          <t>https://leetcode.com/problems/subsets/</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2679,7 +2679,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2689,17 +2689,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Recursion</t>
+          <t>Basic Backtracking</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Power/Exponent</t>
+          <t>Permutations</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Pow(x, n)</t>
+          <t>Permutations</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/powx-n/</t>
+          <t>https://leetcode.com/problems/permutations/</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2729,7 +2729,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2739,22 +2739,22 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Mathematics</t>
+          <t>Basic Backtracking</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Digit Sum</t>
+          <t>Combination</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Add Digits</t>
+          <t>Combination Sum</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2764,7 +2764,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/add-digits/</t>
+          <t>https://leetcode.com/problems/combination-sum/</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2789,22 +2789,22 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Basic Backtracking</t>
+          <t>Stack</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Subsets</t>
+          <t>Validity Check</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Subsets</t>
+          <t>Valid Parentheses</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2814,12 +2814,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/subsets/</t>
+          <t>https://leetcode.com/problems/valid-parentheses/</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2829,7 +2829,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2839,17 +2839,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Basic Backtracking</t>
+          <t>Stack</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Permutations</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Permutations</t>
+          <t>Min Stack</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2864,12 +2864,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/permutations/</t>
+          <t>https://leetcode.com/problems/min-stack/</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2879,7 +2879,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2889,17 +2889,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Basic Backtracking</t>
+          <t>Stack</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Combination</t>
+          <t>Evaluation</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Combination Sum</t>
+          <t>Evaluate Reverse Polish Notation</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/combination-sum/</t>
+          <t>https://leetcode.com/problems/evaluate-reverse-polish-notation/</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2944,17 +2944,17 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Validity Check</t>
+          <t>Monotonic Stack</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Valid Parentheses</t>
+          <t>Daily Temperatures</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2964,12 +2964,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/valid-parentheses/</t>
+          <t>https://leetcode.com/problems/daily-temperatures/</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -2979,7 +2979,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2994,12 +2994,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Path Simplification</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Min Stack</t>
+          <t>Simplify Path</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -3014,12 +3014,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/min-stack/</t>
+          <t>https://leetcode.com/problems/simplify-path/</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3029,7 +3029,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3039,22 +3039,22 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Stack</t>
+          <t>Queue</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Evaluation</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Evaluate Reverse Polish Notation</t>
+          <t>Implement Queue using Stacks</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/evaluate-reverse-polish-notation/</t>
+          <t>https://leetcode.com/problems/implement-queue-using-stacks/</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -3089,37 +3089,37 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Stack</t>
+          <t>Number Theory</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Monotonic Stack</t>
+          <t>Prime Factorization</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Daily Temperatures</t>
+          <t>Prime Factors of a Number</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy-Medium</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/daily-temperatures/</t>
+          <t>https://www.geeksforgeeks.org/prime-factor/</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3129,7 +3129,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3139,17 +3139,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Stack</t>
+          <t>Queue</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Path Simplification</t>
+          <t>Sliding Window</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Simplify Path</t>
+          <t>Sliding Window Maximum</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -3164,7 +3164,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/simplify-path/</t>
+          <t>https://leetcode.com/problems/sliding-window-maximum/</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -3179,7 +3179,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3189,17 +3189,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Queue</t>
+          <t>Linked List</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Reversal</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Implement Queue using Stacks</t>
+          <t>Reverse Linked List</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -3214,12 +3214,12 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/implement-queue-using-stacks/</t>
+          <t>https://leetcode.com/problems/reverse-linked-list/</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3229,7 +3229,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3239,32 +3239,32 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Number Theory</t>
+          <t>Linked List</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Prime Factorization</t>
+          <t>Two Pointer</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Prime Factors of a Number</t>
+          <t>Middle of the Linked List</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Easy-Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/prime-factor/</t>
+          <t>https://leetcode.com/problems/middle-of-the-linked-list/</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -3289,22 +3289,22 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Queue</t>
+          <t>Linked List</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Sliding Window</t>
+          <t>Cycle Detection</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Sliding Window Maximum</t>
+          <t>Linked List Cycle</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -3314,12 +3314,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/sliding-window-maximum/</t>
+          <t>https://leetcode.com/problems/linked-list-cycle/</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3329,7 +3329,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3344,12 +3344,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Reversal</t>
+          <t>Merge</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Reverse Linked List</t>
+          <t>Merge Two Sorted Lists</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/reverse-linked-list/</t>
+          <t>https://leetcode.com/problems/merge-two-sorted-lists/</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -3394,17 +3394,17 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Two Pointer</t>
+          <t>Removal</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Middle of the Linked List</t>
+          <t>Remove Nth Node From End of List</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -3414,12 +3414,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/middle-of-the-linked-list/</t>
+          <t>https://leetcode.com/problems/remove-nth-node-from-end-of-list/</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3444,12 +3444,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Cycle Detection</t>
+          <t>Palindrome Check</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Linked List Cycle</t>
+          <t>Palindrome Linked List</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3464,12 +3464,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/linked-list-cycle/</t>
+          <t>https://leetcode.com/problems/palindrome-linked-list/</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -3479,7 +3479,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3494,12 +3494,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Merge</t>
+          <t>Intersection</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Merge Two Sorted Lists</t>
+          <t>Intersection of Two Linked Lists</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3514,12 +3514,12 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/merge-two-sorted-lists/</t>
+          <t>https://leetcode.com/problems/intersection-of-two-linked-lists/</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -3529,7 +3529,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3539,22 +3539,22 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Linked List</t>
+          <t>Trees</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Removal</t>
+          <t>Traversal</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Remove Nth Node From End of List</t>
+          <t>Maximum Depth of Binary Tree</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3564,12 +3564,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/remove-nth-node-from-end-of-list/</t>
+          <t>https://leetcode.com/problems/maximum-depth-of-binary-tree/</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3579,7 +3579,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3589,22 +3589,22 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Linked List</t>
+          <t>Trees</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Palindrome Check</t>
+          <t>BFS</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Palindrome Linked List</t>
+          <t>Binary Tree Level Order Traversal</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3614,12 +3614,12 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/palindrome-linked-list/</t>
+          <t>https://leetcode.com/problems/binary-tree-level-order-traversal/</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3629,7 +3629,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3639,22 +3639,22 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Linked List</t>
+          <t>Trees</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Intersection</t>
+          <t>Diameter</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Intersection of Two Linked Lists</t>
+          <t>Diameter of Binary Tree</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Easy-Medium</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/intersection-of-two-linked-lists/</t>
+          <t>https://leetcode.com/problems/diameter-of-binary-tree/</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -3694,12 +3694,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Traversal</t>
+          <t>Recursion</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Maximum Depth of Binary Tree</t>
+          <t>Invert Binary Tree</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3714,12 +3714,12 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/maximum-depth-of-binary-tree/</t>
+          <t>https://leetcode.com/problems/invert-binary-tree/</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -3729,7 +3729,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3744,42 +3744,42 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>BFS</t>
+          <t>Symmetry Check</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Binary Tree Level Order Traversal</t>
+          <t>Symmetric Tree</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>LeetCode</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/problems/symmetric-tree/</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Similar</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
           <t>Medium</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>LeetCode</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/problems/binary-tree-level-order-traversal/</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>Community Report</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>High</t>
         </is>
       </c>
     </row>
@@ -3794,17 +3794,17 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Diameter</t>
+          <t>Path Sum</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Diameter of Binary Tree</t>
+          <t>Path Sum</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Easy-Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3814,7 +3814,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/diameter-of-binary-tree/</t>
+          <t>https://leetcode.com/problems/path-sum/</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -3839,22 +3839,22 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Trees</t>
+          <t>Binary Search Trees</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Recursion</t>
+          <t>Validation</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Invert Binary Tree</t>
+          <t>Validate Binary Search Tree</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/invert-binary-tree/</t>
+          <t>https://leetcode.com/problems/validate-binary-search-tree/</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3889,22 +3889,22 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Trees</t>
+          <t>Binary Search Trees</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Symmetry Check</t>
+          <t>Lowest Common Ancestor</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Symmetric Tree</t>
+          <t>Lowest Common Ancestor of a Binary Search Tree</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Easy-Medium</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3914,7 +3914,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/symmetric-tree/</t>
+          <t>https://leetcode.com/problems/lowest-common-ancestor-of-a-binary-search-tree/</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -3939,17 +3939,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Trees</t>
+          <t>Pattern-based Logic</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Path Sum</t>
+          <t>Pattern Printing</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Path Sum</t>
+          <t>Star / Number Pattern Printing</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3959,17 +3959,17 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/path-sum/</t>
+          <t>https://www.geeksforgeeks.org/printing-patterns-using-loops/</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -3979,7 +3979,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3989,22 +3989,22 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Binary Search Trees</t>
+          <t>Heap / Priority Queue</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Validation</t>
+          <t>Kth Largest</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Validate Binary Search Tree</t>
+          <t>Kth Largest Element in a Stream</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/validate-binary-search-tree/</t>
+          <t>https://leetcode.com/problems/kth-largest-element-in-a-stream/</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -4039,22 +4039,22 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Binary Search Trees</t>
+          <t>Heap / Priority Queue</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Lowest Common Ancestor</t>
+          <t>Merge</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Lowest Common Ancestor of a Binary Search Tree</t>
+          <t>Merge k Sorted Lists</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Easy-Medium</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/lowest-common-ancestor-of-a-binary-search-tree/</t>
+          <t>https://leetcode.com/problems/merge-k-sorted-lists/</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -4079,7 +4079,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -4089,37 +4089,37 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Pattern-based Logic</t>
+          <t>Heap / Priority Queue</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Pattern Printing</t>
+          <t>Top K</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Star / Number Pattern Printing</t>
+          <t>Top K Frequent Words</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/printing-patterns-using-loops/</t>
+          <t>https://leetcode.com/problems/top-k-frequent-words/</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -4129,7 +4129,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -4139,22 +4139,22 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Heap / Priority Queue</t>
+          <t>Greedy Algorithms</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Kth Largest</t>
+          <t>Jump Game</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Kth Largest Element in a Stream</t>
+          <t>Jump Game</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -4164,7 +4164,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/kth-largest-element-in-a-stream/</t>
+          <t>https://leetcode.com/problems/jump-game/</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -4189,17 +4189,17 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Heap / Priority Queue</t>
+          <t>Greedy Algorithms</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Merge</t>
+          <t>Interval Scheduling</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Merge k Sorted Lists</t>
+          <t>Non-overlapping Intervals</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/merge-k-sorted-lists/</t>
+          <t>https://leetcode.com/problems/non-overlapping-intervals/</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -4229,7 +4229,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -4239,22 +4239,22 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Heap / Priority Queue</t>
+          <t>Simulation</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Top K</t>
+          <t>Grid Simulation</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Top K Frequent Words</t>
+          <t>Robot Return to Origin</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/top-k-frequent-words/</t>
+          <t>https://leetcode.com/problems/robot-return-to-origin/</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -4289,22 +4289,22 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Greedy Algorithms</t>
+          <t>Dynamic Programming</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Jump Game</t>
+          <t>1D DP</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Jump Game</t>
+          <t>Climbing Stairs</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -4314,12 +4314,12 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/jump-game/</t>
+          <t>https://leetcode.com/problems/climbing-stairs/</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -4329,7 +4329,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -4339,17 +4339,17 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Greedy Algorithms</t>
+          <t>Dynamic Programming</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Interval Scheduling</t>
+          <t>1D DP</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Non-overlapping Intervals</t>
+          <t>House Robber</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -4364,12 +4364,12 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/non-overlapping-intervals/</t>
+          <t>https://leetcode.com/problems/house-robber/</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -4379,7 +4379,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -4389,22 +4389,22 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Simulation</t>
+          <t>Dynamic Programming</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Grid Simulation</t>
+          <t>Coin Change</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Robot Return to Origin</t>
+          <t>Coin Change</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/robot-return-to-origin/</t>
+          <t>https://leetcode.com/problems/coin-change/</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -4444,17 +4444,17 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>1D DP</t>
+          <t>Subsequence</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Climbing Stairs</t>
+          <t>Longest Increasing Subsequence</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -4464,12 +4464,12 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/climbing-stairs/</t>
+          <t>https://leetcode.com/problems/longest-increasing-subsequence/</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -4479,7 +4479,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -4489,22 +4489,22 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Dynamic Programming</t>
+          <t>Graph Basics</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>1D DP</t>
+          <t>Flood Fill</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>House Robber</t>
+          <t>Flood Fill</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/house-robber/</t>
+          <t>https://leetcode.com/problems/flood-fill/</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -4539,17 +4539,17 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Dynamic Programming</t>
+          <t>Graph Basics</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Coin Change</t>
+          <t>Islands / DFS</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Coin Change</t>
+          <t>Number of Islands</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -4564,12 +4564,12 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/coin-change/</t>
+          <t>https://leetcode.com/problems/number-of-islands/</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -4579,7 +4579,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -4589,17 +4589,17 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Dynamic Programming</t>
+          <t>Graph Basics</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Subsequence</t>
+          <t>BFS</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Longest Increasing Subsequence</t>
+          <t>Rotting Oranges</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/longest-increasing-subsequence/</t>
+          <t>https://leetcode.com/problems/rotting-oranges/</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -4644,17 +4644,17 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Flood Fill</t>
+          <t>DFS</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Flood Fill</t>
+          <t>Clone Graph</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -4664,12 +4664,12 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/flood-fill/</t>
+          <t>https://leetcode.com/problems/clone-graph/</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -4679,7 +4679,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -4689,22 +4689,22 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Graph Basics</t>
+          <t>Mathematics</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Islands / DFS</t>
+          <t>Number Reversal</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Number of Islands</t>
+          <t>Palindrome Number</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/number-of-islands/</t>
+          <t>https://leetcode.com/problems/palindrome-number/</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -4739,22 +4739,22 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Graph Basics</t>
+          <t>Bit Manipulation</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>BFS</t>
+          <t>Bit Counting DP</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Rotting Oranges</t>
+          <t>Counting Bits</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/rotting-oranges/</t>
+          <t>https://leetcode.com/problems/counting-bits/</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -4779,7 +4779,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -4789,17 +4789,17 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Graph Basics</t>
+          <t>Number Theory</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>DFS</t>
+          <t>Sieve of Eratosthenes</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Clone Graph</t>
+          <t>Count Primes</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4814,12 +4814,12 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/clone-graph/</t>
+          <t>https://leetcode.com/problems/count-primes/</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Similar</t>
+          <t>Community Report</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -4829,7 +4829,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -4839,17 +4839,17 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Mathematics</t>
+          <t>Miscellaneous</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Number Reversal</t>
+          <t>String Math</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Palindrome Number</t>
+          <t>Greatest Common Divisor of Strings</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -4864,12 +4864,12 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/palindrome-number/</t>
+          <t>https://leetcode.com/problems/greatest-common-divisor-of-strings/</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>Community Report</t>
+          <t>Similar</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -4879,160 +4879,13 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="15.75" customHeight="1">
-      <c r="A89" t="n">
-        <v>88</v>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>Bit Manipulation</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>Bit Counting DP</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr">
-        <is>
-          <t>Counting Bits</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>LeetCode</t>
-        </is>
-      </c>
-      <c r="G89" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/problems/counting-bits/</t>
-        </is>
-      </c>
-      <c r="H89" t="inlineStr">
-        <is>
-          <t>Similar</t>
-        </is>
-      </c>
-      <c r="I89" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J89" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-    </row>
-    <row r="90" ht="15.75" customHeight="1">
-      <c r="A90" t="n">
-        <v>89</v>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>Number Theory</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>Sieve of Eratosthenes</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>Count Primes</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>LeetCode</t>
-        </is>
-      </c>
-      <c r="G90" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/problems/count-primes/</t>
-        </is>
-      </c>
-      <c r="H90" t="inlineStr">
-        <is>
-          <t>Community Report</t>
-        </is>
-      </c>
-      <c r="I90" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J90" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" ht="15.75" customHeight="1">
-      <c r="A91" t="n">
-        <v>90</v>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>Miscellaneous</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>String Math</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>Greatest Common Divisor of Strings</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>LeetCode</t>
-        </is>
-      </c>
-      <c r="G91" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/problems/greatest-common-divisor-of-strings/</t>
-        </is>
-      </c>
-      <c r="H91" t="inlineStr">
-        <is>
-          <t>Similar</t>
-        </is>
-      </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J91" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
+    </row>
+    <row r="89" ht="15.75" customHeight="1"/>
+    <row r="90" ht="15.75" customHeight="1"/>
+    <row r="91" ht="15.75" customHeight="1"/>
     <row r="92" ht="15.75" customHeight="1"/>
     <row r="93" ht="15.75" customHeight="1"/>
     <row r="94" ht="15.75" customHeight="1"/>

</xml_diff>